<commit_message>
Arreglada lógica de iconos, revisión diseño.
</commit_message>
<xml_diff>
--- a/datosfinales.xlsx
+++ b/datosfinales.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$O$848</definedName>
@@ -653,7 +653,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -702,7 +702,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -751,7 +751,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -845,7 +845,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -935,7 +935,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G21" s="2" t="n"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G23" s="2" t="n"/>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G25" s="2" t="n"/>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G36" s="2" t="n"/>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G41" s="2" t="n"/>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G43" s="2" t="n"/>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>2025-02-04</t>
+          <t>404</t>
         </is>
       </c>
       <c r="G44" s="3" t="n"/>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G46" s="3" t="n"/>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G47" s="3" t="n"/>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G48" s="3" t="n"/>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G49" s="3" t="n"/>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G52" s="3" t="n"/>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="G53" s="3" t="n"/>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G58" s="3" t="n"/>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G59" s="3" t="n"/>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G60" s="3" t="n"/>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G61" s="3" t="n"/>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G64" s="3" t="n"/>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G66" s="3" t="n"/>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G68" s="4" t="n"/>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G72" s="4" t="n"/>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G78" s="4" t="n"/>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G84" s="4" t="n"/>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G95" s="4" t="n"/>
@@ -5445,7 +5445,7 @@
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G104" s="4" t="n"/>
@@ -5837,7 +5837,7 @@
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G112" s="4" t="n"/>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G136" s="4" t="n"/>
@@ -7421,7 +7421,7 @@
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>2025-11-24</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="G144" s="4" t="n"/>
@@ -8160,7 +8160,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G159" s="4" t="n"/>
@@ -8315,7 +8315,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>2025-10-22</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G162" s="4" t="n"/>
@@ -9291,7 +9291,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="G182" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
       </c>
       <c r="F185" s="4" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G185" s="4" t="n"/>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="F189" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G189" s="4" t="n"/>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="F191" s="4" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G191" s="4" t="n"/>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="F192" s="4" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="G192" s="4" t="n"/>
@@ -10621,7 +10621,7 @@
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G208" s="4" t="n"/>
@@ -10976,7 +10976,7 @@
       </c>
       <c r="F215" s="4" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G215" s="4" t="n"/>
@@ -11176,7 +11176,7 @@
       </c>
       <c r="F219" s="4" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="G219" s="4" t="n"/>
@@ -11833,7 +11833,7 @@
       </c>
       <c r="F232" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G232" s="4" t="n"/>
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F243" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G243" s="4" t="n"/>
@@ -12486,7 +12486,7 @@
       </c>
       <c r="F245" s="4" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G245" s="4" t="n"/>
@@ -12539,7 +12539,7 @@
       </c>
       <c r="F246" s="4" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G246" s="4" t="n"/>
@@ -12637,7 +12637,7 @@
       </c>
       <c r="F248" s="4" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G248" s="4" t="n"/>
@@ -12743,7 +12743,7 @@
       </c>
       <c r="F250" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G250" s="4" t="n"/>
@@ -12955,7 +12955,7 @@
       </c>
       <c r="F254" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G254" s="4" t="n"/>
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F287" s="4" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G287" s="4" t="n"/>
@@ -14743,7 +14743,7 @@
       </c>
       <c r="F290" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G290" s="4" t="n"/>
@@ -15282,7 +15282,7 @@
       </c>
       <c r="F301" s="4" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G301" s="4" t="n"/>
@@ -15694,7 +15694,7 @@
       </c>
       <c r="F309" s="4" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G309" s="4" t="n"/>
@@ -15935,7 +15935,7 @@
       </c>
       <c r="F314" s="4" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G314" s="4" t="n"/>
@@ -16274,7 +16274,7 @@
       </c>
       <c r="F321" s="4" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="G321" s="4" t="n"/>
@@ -16486,7 +16486,7 @@
       </c>
       <c r="F325" s="4" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>404</t>
         </is>
       </c>
       <c r="G325" s="4" t="n"/>
@@ -16792,7 +16792,7 @@
       </c>
       <c r="F331" s="4" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="G331" s="4" t="n"/>
@@ -16898,7 +16898,7 @@
       </c>
       <c r="F333" s="4" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G333" s="4" t="n"/>
@@ -17053,7 +17053,7 @@
       </c>
       <c r="F336" s="4" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="G336" s="4" t="n"/>
@@ -17159,7 +17159,7 @@
       </c>
       <c r="F338" s="4" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="G338" s="4" t="n"/>
@@ -18460,7 +18460,7 @@
       </c>
       <c r="F363" s="4" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="G363" s="4" t="n"/>
@@ -18566,7 +18566,7 @@
       </c>
       <c r="F365" s="4" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G365" s="4" t="n"/>
@@ -19023,7 +19023,7 @@
       </c>
       <c r="F374" s="4" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G374" s="4" t="n"/>
@@ -19235,7 +19235,7 @@
       </c>
       <c r="F378" s="4" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G378" s="4" t="n"/>
@@ -19476,7 +19476,7 @@
       </c>
       <c r="F383" s="4" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="G383" s="4" t="n"/>
@@ -19631,7 +19631,7 @@
       </c>
       <c r="F386" s="4" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G386" s="4" t="n"/>
@@ -20880,7 +20880,7 @@
       </c>
       <c r="F411" s="4" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="G411" s="4" t="n"/>
@@ -21908,7 +21908,7 @@
       </c>
       <c r="F435" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G435" s="5" t="n"/>
@@ -21961,7 +21961,7 @@
       </c>
       <c r="F436" s="5" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G436" s="5" t="n"/>
@@ -23679,7 +23679,7 @@
       </c>
       <c r="F478" s="5" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="G478" s="5" t="n"/>
@@ -24450,7 +24450,7 @@
       </c>
       <c r="F497" s="5" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="G497" s="5" t="n"/>
@@ -24618,7 +24618,7 @@
       </c>
       <c r="F501" s="5" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="G501" s="5" t="n"/>
@@ -25062,7 +25062,7 @@
       </c>
       <c r="F513" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="G513" s="5" t="n"/>
@@ -25431,7 +25431,7 @@
       </c>
       <c r="F522" s="5" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="G522" s="5" t="n"/>
@@ -25521,7 +25521,7 @@
       </c>
       <c r="F524" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G524" s="5" t="n"/>
@@ -25948,7 +25948,7 @@
       </c>
       <c r="F535" s="5" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="G535" s="5" t="n"/>
@@ -26559,7 +26559,7 @@
       </c>
       <c r="F550" s="5" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="G550" s="5" t="n"/>
@@ -27962,7 +27962,7 @@
       </c>
       <c r="F585" s="5" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>404</t>
         </is>
       </c>
       <c r="G585" s="5" t="n"/>
@@ -28788,7 +28788,7 @@
       </c>
       <c r="F607" s="5" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G607" s="5" t="n"/>
@@ -29103,7 +29103,7 @@
       </c>
       <c r="F614" s="5" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="G614" s="5" t="n"/>
@@ -29444,7 +29444,7 @@
       </c>
       <c r="F623" s="5" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="G623" s="5" t="n"/>
@@ -29953,7 +29953,7 @@
       </c>
       <c r="F636" s="5" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G636" s="5" t="n"/>
@@ -30064,7 +30064,7 @@
       </c>
       <c r="F639" s="5" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="G639" s="5" t="n"/>
@@ -31294,7 +31294,7 @@
       </c>
       <c r="F669" s="5" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="G669" s="5" t="n"/>
@@ -31828,7 +31828,7 @@
       </c>
       <c r="F683" s="5" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G683" s="5" t="n"/>
@@ -31873,7 +31873,7 @@
       </c>
       <c r="F684" s="5" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G684" s="5" t="n"/>
@@ -33103,7 +33103,7 @@
       </c>
       <c r="F714" s="6" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G714" s="6" t="n"/>
@@ -33185,7 +33185,7 @@
       </c>
       <c r="F716" s="6" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G716" s="6" t="n"/>
@@ -33230,7 +33230,7 @@
       </c>
       <c r="F717" s="6" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="G717" s="6" t="n"/>
@@ -33320,7 +33320,7 @@
       </c>
       <c r="F719" s="6" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G719" s="6" t="n"/>
@@ -33484,7 +33484,7 @@
       </c>
       <c r="F723" s="6" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G723" s="6" t="n"/>
@@ -33529,7 +33529,7 @@
       </c>
       <c r="F724" s="6" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G724" s="6" t="inlineStr">
@@ -33539,7 +33539,7 @@
       </c>
       <c r="H724" s="6" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="I724" s="6" t="inlineStr">
@@ -33627,7 +33627,7 @@
       </c>
       <c r="F726" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G726" s="6" t="n"/>
@@ -33672,7 +33672,7 @@
       </c>
       <c r="F727" s="6" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G727" s="6" t="n"/>
@@ -33717,7 +33717,7 @@
       </c>
       <c r="F728" s="6" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G728" s="6" t="n"/>
@@ -35031,7 +35031,7 @@
       </c>
       <c r="F758" s="7" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G758" s="7" t="n"/>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="F792" s="7" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="G792" s="7" t="n"/>
@@ -37004,7 +37004,7 @@
       </c>
       <c r="F799" s="8" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G799" s="8" t="n"/>
@@ -37098,7 +37098,7 @@
       </c>
       <c r="F801" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G801" s="8" t="n"/>
@@ -37315,7 +37315,7 @@
       </c>
       <c r="F806" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G806" s="8" t="n"/>
@@ -37405,7 +37405,7 @@
       </c>
       <c r="F808" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G808" s="8" t="n"/>
@@ -37499,7 +37499,7 @@
       </c>
       <c r="F810" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G810" s="8" t="n"/>
@@ -37597,7 +37597,7 @@
       </c>
       <c r="F812" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G812" s="8" t="n"/>
@@ -37781,7 +37781,7 @@
       </c>
       <c r="F816" s="8" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G816" s="8" t="n"/>
@@ -37875,7 +37875,7 @@
       </c>
       <c r="F818" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G818" s="8" t="n"/>
@@ -37965,7 +37965,7 @@
       </c>
       <c r="F820" s="8" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G820" s="8" t="n"/>
@@ -38063,7 +38063,7 @@
       </c>
       <c r="F822" s="8" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G822" s="8" t="n"/>
@@ -38198,7 +38198,7 @@
       </c>
       <c r="F825" s="8" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G825" s="8" t="n"/>
@@ -38288,7 +38288,7 @@
       </c>
       <c r="F827" s="8" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G827" s="8" t="n"/>
@@ -38337,7 +38337,7 @@
       </c>
       <c r="F828" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G828" s="8" t="n"/>
@@ -38386,7 +38386,7 @@
       </c>
       <c r="F829" s="8" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G829" s="8" t="n"/>
@@ -38480,7 +38480,7 @@
       </c>
       <c r="F831" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G831" s="8" t="n"/>
@@ -38529,7 +38529,7 @@
       </c>
       <c r="F832" s="8" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="G832" s="8" t="n"/>
@@ -38578,7 +38578,7 @@
       </c>
       <c r="F833" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G833" s="8" t="n"/>
@@ -38627,7 +38627,7 @@
       </c>
       <c r="F834" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G834" s="8" t="n"/>
@@ -38676,7 +38676,7 @@
       </c>
       <c r="F835" s="8" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G835" s="8" t="n"/>
@@ -38725,7 +38725,7 @@
       </c>
       <c r="F836" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="G836" s="8" t="n"/>
@@ -38774,7 +38774,7 @@
       </c>
       <c r="F837" s="8" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G837" s="8" t="n"/>
@@ -38823,7 +38823,7 @@
       </c>
       <c r="F838" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G838" s="8" t="n"/>
@@ -38872,7 +38872,7 @@
       </c>
       <c r="F839" s="8" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G839" s="8" t="n"/>
@@ -39015,7 +39015,7 @@
       </c>
       <c r="F842" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G842" s="8" t="n"/>
@@ -39064,7 +39064,7 @@
       </c>
       <c r="F843" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G843" s="8" t="n"/>
@@ -39113,7 +39113,7 @@
       </c>
       <c r="F844" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G844" s="8" t="n"/>
@@ -39162,7 +39162,7 @@
       </c>
       <c r="F845" s="8" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G845" s="8" t="n"/>
@@ -39211,7 +39211,7 @@
       </c>
       <c r="F846" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G846" s="8" t="n"/>
@@ -39260,7 +39260,7 @@
       </c>
       <c r="F847" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="G847" s="8" t="n"/>
@@ -39309,7 +39309,7 @@
       </c>
       <c r="F848" s="8" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G848" s="8" t="n"/>

</xml_diff>